<commit_message>
Estadísticas: leer Excel de competencias y mostrar nivel que puede presentar en Normativos
- xlsx-reader: nueva función readSheetInfo (filas + celdas combinadas).
- Estadísticas lee 'Estadistica de competencias totales.xlsx' (Drive, con data.json de respaldo).
- Vista Normativos: lista de atletas desde Normativos, resumen 'Puede presentar hasta…'
  por aparato y columna 'Necesario' (barras de nivel AG–AO del Excel).
- Ajuste de anchos de la tabla de 3 columnas y color del resumen de nivel.
- NORMATIVOS_AKC.xlsx: fórmulas de FICHA/CONSOLIDADO/INDICADORES cuentan N/A como no adquirido
  (la hoja NORMATIVOS no cambia).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EsLdurz1dkmzTgP9Dw2L4J
</commit_message>
<xml_diff>
--- a/modulos/normativos/NORMATIVOS_AKC.xlsx
+++ b/modulos/normativos/NORMATIVOS_AKC.xlsx
@@ -19,7 +19,7 @@
     <sheet name="CONSOLIDADO" sheetId="3" r:id="rId4"/>
     <sheet name="CATALOGOS" sheetId="2" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029" forceFullCalc="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -939,7 +939,7 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>N/A = no aplica / aún no corresponde</t>
+    <t>N/A = No adquirido: no lo hizo, no le sale, le faltó aprenderlo</t>
   </si>
   <si>
     <t>ACROBATICO HACÍA DELANTE</t>
@@ -1101,7 +1101,7 @@
     <t>Elementos en proceso</t>
   </si>
   <si>
-    <t>DOMINIO PROMEDIO POR APARATO</t>
+    <t>DOMINIO POR APARATO (ATLETA SELECCIONADO EN FICHA)</t>
   </si>
   <si>
     <t xml:space="preserve">Consolidado = 🟩
@@ -31698,8 +31698,8 @@
         <v>0</v>
       </c>
       <c r="H6" s="13">
-        <f t="shared" ref="H6:H21" si="0">IFERROR(E6/(E6+F6+G6),0)</f>
-        <v>1</v>
+        <f>IFERROR(E6/COUNTA(NORMATIVOS!$B$3:$B$16),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -31726,8 +31726,8 @@
         <v>0</v>
       </c>
       <c r="H7" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E7/COUNTA(NORMATIVOS!$B$17:$B$27),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -31754,8 +31754,8 @@
         <v>0</v>
       </c>
       <c r="H8" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E8/COUNTA(NORMATIVOS!$B$28:$B$37),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -31782,8 +31782,8 @@
         <v>0</v>
       </c>
       <c r="H9" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E9/COUNTA(NORMATIVOS!$B$38:$B$46),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -31810,8 +31810,8 @@
         <v>0</v>
       </c>
       <c r="H10" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E10/COUNTA(NORMATIVOS!$B$49:$B$64),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -31820,7 +31820,7 @@
       </c>
       <c r="B11" s="13">
         <f>INDEX(CONSOLIDADO!$G$4:$G$1048576,MATCH($B$3,CONSOLIDADO!$A$4:$A$1048576,0))</f>
-        <v>0.87984496124031009</v>
+        <v>0.850187265917603</v>
       </c>
       <c r="D11" t="s">
         <v>99</v>
@@ -31838,8 +31838,8 @@
         <v>0</v>
       </c>
       <c r="H11" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E11/COUNTA(NORMATIVOS!$B$65:$B$78),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -31847,20 +31847,20 @@
         <v>109</v>
       </c>
       <c r="E12">
-        <f>--(INDEX(NORMATIVOS!$C$79:$XFD$79,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$80:$XFD$80,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$81:$XFD$81,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$82:$XFD$82,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$83:$XFD$83,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$84:$XFD$84,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$85:$XFD$85,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$86:$XFD$86,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$87:$XFD$87,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$88:$XFD$88,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$89:$XFD$89,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$90:$XFD$90,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$91:$XFD$91,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$92:$XFD$92,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$93:$XFD$93,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$94:$XFD$94,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$95:$XFD$95,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$96:$XFD$96,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$97:$XFD$97,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$98:$XFD$98,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$99:$XFD$99,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$100:$XFD$100,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$101:$XFD$101,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$103:$XFD$103,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$104:$XFD$104,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$105:$XFD$105,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")</f>
-        <v>23</v>
+        <f>--(INDEX(NORMATIVOS!$C$79:$XFD$79,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$80:$XFD$80,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$81:$XFD$81,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$82:$XFD$82,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$83:$XFD$83,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$84:$XFD$84,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$85:$XFD$85,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$86:$XFD$86,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$87:$XFD$87,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$88:$XFD$88,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$89:$XFD$89,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$90:$XFD$90,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$91:$XFD$91,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$92:$XFD$92,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$93:$XFD$93,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$94:$XFD$94,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$95:$XFD$95,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$96:$XFD$96,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$97:$XFD$97,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$98:$XFD$98,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$99:$XFD$99,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$100:$XFD$100,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$101:$XFD$101,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$102:$XFD$102,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$103:$XFD$103,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$104:$XFD$104,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$105:$XFD$105,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")</f>
+        <v>24</v>
       </c>
       <c r="F12">
-        <f>--(INDEX(NORMATIVOS!$C$79:$XFD$79,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$80:$XFD$80,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$81:$XFD$81,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$82:$XFD$82,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$83:$XFD$83,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$84:$XFD$84,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$85:$XFD$85,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$86:$XFD$86,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$87:$XFD$87,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$88:$XFD$88,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$89:$XFD$89,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$90:$XFD$90,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$91:$XFD$91,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$92:$XFD$92,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$93:$XFD$93,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$94:$XFD$94,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$95:$XFD$95,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$96:$XFD$96,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$97:$XFD$97,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$98:$XFD$98,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$99:$XFD$99,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$100:$XFD$100,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$101:$XFD$101,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$103:$XFD$103,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$104:$XFD$104,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$105:$XFD$105,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")</f>
+        <f>--(INDEX(NORMATIVOS!$C$79:$XFD$79,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$80:$XFD$80,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$81:$XFD$81,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$82:$XFD$82,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$83:$XFD$83,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$84:$XFD$84,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$85:$XFD$85,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$86:$XFD$86,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$87:$XFD$87,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$88:$XFD$88,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$89:$XFD$89,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$90:$XFD$90,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$91:$XFD$91,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$92:$XFD$92,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$93:$XFD$93,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$94:$XFD$94,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$95:$XFD$95,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$96:$XFD$96,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$97:$XFD$97,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$98:$XFD$98,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$99:$XFD$99,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$100:$XFD$100,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$101:$XFD$101,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$102:$XFD$102,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$103:$XFD$103,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$104:$XFD$104,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$105:$XFD$105,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")</f>
         <v>0</v>
       </c>
       <c r="G12">
-        <f>--(INDEX(NORMATIVOS!$C$79:$XFD$79,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$80:$XFD$80,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$81:$XFD$81,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$82:$XFD$82,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$83:$XFD$83,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$84:$XFD$84,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$85:$XFD$85,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$86:$XFD$86,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$87:$XFD$87,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$88:$XFD$88,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$89:$XFD$89,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$90:$XFD$90,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$91:$XFD$91,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$92:$XFD$92,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$93:$XFD$93,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$94:$XFD$94,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$95:$XFD$95,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$96:$XFD$96,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$97:$XFD$97,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$98:$XFD$98,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$99:$XFD$99,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$100:$XFD$100,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$101:$XFD$101,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$103:$XFD$103,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$104:$XFD$104,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$105:$XFD$105,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")</f>
+        <f>--(INDEX(NORMATIVOS!$C$79:$XFD$79,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$80:$XFD$80,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$81:$XFD$81,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$82:$XFD$82,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$83:$XFD$83,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$84:$XFD$84,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$85:$XFD$85,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$86:$XFD$86,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$87:$XFD$87,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$88:$XFD$88,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$89:$XFD$89,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$90:$XFD$90,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$91:$XFD$91,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$92:$XFD$92,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$93:$XFD$93,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$94:$XFD$94,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$95:$XFD$95,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$96:$XFD$96,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$97:$XFD$97,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$98:$XFD$98,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$99:$XFD$99,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$100:$XFD$100,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$101:$XFD$101,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$102:$XFD$102,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$103:$XFD$103,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$104:$XFD$104,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$105:$XFD$105,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")</f>
         <v>3</v>
       </c>
       <c r="H12" s="13">
-        <f t="shared" si="0"/>
-        <v>0.88461538461538458</v>
+        <f>IFERROR(E12/COUNTA(NORMATIVOS!$B$79:$B$105),0)</f>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -31880,8 +31880,8 @@
         <v>2</v>
       </c>
       <c r="H13" s="13">
-        <f t="shared" si="0"/>
-        <v>0.8571428571428571</v>
+        <f>IFERROR(E13/COUNTA(NORMATIVOS!$B$108:$B$122),0)</f>
+        <v>0.8</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -31901,8 +31901,8 @@
         <v>0</v>
       </c>
       <c r="H14" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E14/COUNTA(NORMATIVOS!$B$123:$B$142),0)</f>
+        <v>0.9</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -31922,8 +31922,8 @@
         <v>0</v>
       </c>
       <c r="H15" s="13">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>IFERROR(E15/COUNTA(NORMATIVOS!$B$145:$B$151),0)</f>
+        <v>1.0</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -31943,8 +31943,8 @@
         <v>6</v>
       </c>
       <c r="H16" s="13">
-        <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
+        <f>IFERROR(E16/COUNTA(NORMATIVOS!$B$152:$B$173),0)</f>
+        <v>0.6363636363636364</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -31964,8 +31964,8 @@
         <v>0</v>
       </c>
       <c r="H17" s="13">
-        <f t="shared" si="0"/>
-        <v>0.94444444444444442</v>
+        <f>IFERROR(E17/COUNTA(NORMATIVOS!$B$176:$B$193),0)</f>
+        <v>0.9444444444444444</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -31973,20 +31973,20 @@
         <v>220</v>
       </c>
       <c r="E18">
-        <f>--(INDEX(NORMATIVOS!$C$194:$XFD$194,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$195:$XFD$195,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$196:$XFD$196,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$197:$XFD$197,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$198:$XFD$198,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$199:$XFD$199,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$200:$XFD$200,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$201:$XFD$201,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$202:$XFD$202,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$203:$XFD$203,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$204:$XFD$204,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$205:$XFD$205,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$206:$XFD$206,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$207:$XFD$207,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$209:$XFD$209,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$210:$XFD$210,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$211:$XFD$211,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$212:$XFD$212,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$213:$XFD$213,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$214:$XFD$214,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$215:$XFD$215,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$216:$XFD$216,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$217:$XFD$217,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$218:$XFD$218,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")</f>
-        <v>18</v>
+        <f>--(INDEX(NORMATIVOS!$C$194:$XFD$194,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$195:$XFD$195,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$196:$XFD$196,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$197:$XFD$197,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$198:$XFD$198,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$199:$XFD$199,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$200:$XFD$200,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$201:$XFD$201,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$202:$XFD$202,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$203:$XFD$203,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$204:$XFD$204,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$205:$XFD$205,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$206:$XFD$206,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$207:$XFD$207,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$208:$XFD$208,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$209:$XFD$209,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$210:$XFD$210,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$211:$XFD$211,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$212:$XFD$212,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$213:$XFD$213,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$214:$XFD$214,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$215:$XFD$215,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$216:$XFD$216,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$217:$XFD$217,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$218:$XFD$218,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")</f>
+        <v>19</v>
       </c>
       <c r="F18">
-        <f>--(INDEX(NORMATIVOS!$C$194:$XFD$194,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$195:$XFD$195,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$196:$XFD$196,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$197:$XFD$197,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$198:$XFD$198,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$199:$XFD$199,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$200:$XFD$200,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$201:$XFD$201,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$202:$XFD$202,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$203:$XFD$203,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$204:$XFD$204,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$205:$XFD$205,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$206:$XFD$206,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$207:$XFD$207,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$209:$XFD$209,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$210:$XFD$210,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$211:$XFD$211,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$212:$XFD$212,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$213:$XFD$213,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$214:$XFD$214,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$215:$XFD$215,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$216:$XFD$216,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$217:$XFD$217,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$218:$XFD$218,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")</f>
+        <f>--(INDEX(NORMATIVOS!$C$194:$XFD$194,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$195:$XFD$195,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$196:$XFD$196,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$197:$XFD$197,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$198:$XFD$198,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$199:$XFD$199,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$200:$XFD$200,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$201:$XFD$201,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$202:$XFD$202,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$203:$XFD$203,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$204:$XFD$204,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$205:$XFD$205,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$206:$XFD$206,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$207:$XFD$207,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$208:$XFD$208,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$209:$XFD$209,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$210:$XFD$210,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$211:$XFD$211,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$212:$XFD$212,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$213:$XFD$213,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$214:$XFD$214,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$215:$XFD$215,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$216:$XFD$216,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$217:$XFD$217,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$218:$XFD$218,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")</f>
         <v>3</v>
       </c>
       <c r="G18">
-        <f>--(INDEX(NORMATIVOS!$C$194:$XFD$194,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$195:$XFD$195,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$196:$XFD$196,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$197:$XFD$197,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$198:$XFD$198,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$199:$XFD$199,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$200:$XFD$200,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$201:$XFD$201,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$202:$XFD$202,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$203:$XFD$203,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$204:$XFD$204,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$205:$XFD$205,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$206:$XFD$206,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$207:$XFD$207,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$209:$XFD$209,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$210:$XFD$210,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$211:$XFD$211,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$212:$XFD$212,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$213:$XFD$213,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$214:$XFD$214,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$215:$XFD$215,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$216:$XFD$216,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$217:$XFD$217,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$218:$XFD$218,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")</f>
+        <f>--(INDEX(NORMATIVOS!$C$194:$XFD$194,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$195:$XFD$195,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$196:$XFD$196,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$197:$XFD$197,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$198:$XFD$198,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$199:$XFD$199,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$200:$XFD$200,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$201:$XFD$201,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$202:$XFD$202,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$203:$XFD$203,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$204:$XFD$204,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$205:$XFD$205,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$206:$XFD$206,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$207:$XFD$207,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$208:$XFD$208,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$209:$XFD$209,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$210:$XFD$210,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$211:$XFD$211,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$212:$XFD$212,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$213:$XFD$213,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$214:$XFD$214,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$215:$XFD$215,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$216:$XFD$216,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$217:$XFD$217,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$218:$XFD$218,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")</f>
         <v>2</v>
       </c>
       <c r="H18" s="13">
-        <f t="shared" si="0"/>
-        <v>0.78260869565217395</v>
+        <f>IFERROR(E18/COUNTA(NORMATIVOS!$B$194:$B$218),0)</f>
+        <v>0.76</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -32006,8 +32006,8 @@
         <v>3</v>
       </c>
       <c r="H19" s="13">
-        <f t="shared" si="0"/>
-        <v>0.63636363636363635</v>
+        <f>IFERROR(E19/COUNTA(NORMATIVOS!$B$219:$B$231),0)</f>
+        <v>0.5384615384615384</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -32027,8 +32027,8 @@
         <v>5</v>
       </c>
       <c r="H20" s="13">
-        <f t="shared" si="0"/>
-        <v>0.76923076923076927</v>
+        <f>IFERROR(E20/COUNTA(NORMATIVOS!$B$234:$B$261),0)</f>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -32036,20 +32036,20 @@
         <v>278</v>
       </c>
       <c r="E21">
-        <f>--(INDEX(NORMATIVOS!$C$262:$XFD$262,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$263:$XFD$263,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$264:$XFD$264,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$266:$XFD$266,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$267:$XFD$267,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$268:$XFD$268,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$269:$XFD$269,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$270:$XFD$270,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$271:$XFD$271,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$272:$XFD$272,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$273:$XFD$273,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$274:$XFD$274,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$275:$XFD$275,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$276:$XFD$276,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$277:$XFD$277,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$278:$XFD$278,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$279:$XFD$279,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")</f>
-        <v>14</v>
+        <f>--(INDEX(NORMATIVOS!$C$262:$XFD$262,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$263:$XFD$263,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$264:$XFD$264,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$265:$XFD$265,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$266:$XFD$266,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$267:$XFD$267,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$268:$XFD$268,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$269:$XFD$269,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$270:$XFD$270,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$271:$XFD$271,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$272:$XFD$272,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$273:$XFD$273,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$274:$XFD$274,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$275:$XFD$275,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$276:$XFD$276,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$277:$XFD$277,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$278:$XFD$278,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")+--(INDEX(NORMATIVOS!$C$279:$XFD$279,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Consolidado")</f>
+        <v>15</v>
       </c>
       <c r="F21">
-        <f>--(INDEX(NORMATIVOS!$C$262:$XFD$262,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$263:$XFD$263,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$264:$XFD$264,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$266:$XFD$266,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$267:$XFD$267,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$268:$XFD$268,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$269:$XFD$269,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$270:$XFD$270,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$271:$XFD$271,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$272:$XFD$272,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$273:$XFD$273,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$274:$XFD$274,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$275:$XFD$275,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$276:$XFD$276,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$277:$XFD$277,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$278:$XFD$278,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$279:$XFD$279,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")</f>
+        <f>--(INDEX(NORMATIVOS!$C$262:$XFD$262,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$263:$XFD$263,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$264:$XFD$264,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$265:$XFD$265,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$266:$XFD$266,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$267:$XFD$267,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$268:$XFD$268,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$269:$XFD$269,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$270:$XFD$270,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$271:$XFD$271,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$272:$XFD$272,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$273:$XFD$273,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$274:$XFD$274,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$275:$XFD$275,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$276:$XFD$276,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$277:$XFD$277,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$278:$XFD$278,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")+--(INDEX(NORMATIVOS!$C$279:$XFD$279,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="En proceso")</f>
         <v>0</v>
       </c>
       <c r="G21">
-        <f>--(INDEX(NORMATIVOS!$C$262:$XFD$262,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$263:$XFD$263,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$264:$XFD$264,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$266:$XFD$266,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$267:$XFD$267,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$268:$XFD$268,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$269:$XFD$269,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$270:$XFD$270,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$271:$XFD$271,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$272:$XFD$272,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$273:$XFD$273,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$274:$XFD$274,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$275:$XFD$275,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$276:$XFD$276,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$277:$XFD$277,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$278:$XFD$278,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$279:$XFD$279,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")</f>
+        <f>--(INDEX(NORMATIVOS!$C$262:$XFD$262,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$263:$XFD$263,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$264:$XFD$264,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$265:$XFD$265,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$266:$XFD$266,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$267:$XFD$267,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$268:$XFD$268,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$269:$XFD$269,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$270:$XFD$270,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$271:$XFD$271,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$272:$XFD$272,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$273:$XFD$273,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$274:$XFD$274,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$275:$XFD$275,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$276:$XFD$276,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$277:$XFD$277,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$278:$XFD$278,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")+--(INDEX(NORMATIVOS!$C$279:$XFD$279,1,MATCH($B$3,NORMATIVOS!$C$1:$XFD$1,0))="Proyección")</f>
         <v>3</v>
       </c>
       <c r="H21" s="13">
-        <f t="shared" si="0"/>
-        <v>0.82352941176470584</v>
+        <f>IFERROR(E21/COUNTA(NORMATIVOS!$B$262:$B$279),0)</f>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -35359,7 +35359,7 @@
       </c>
       <c r="B4" s="15">
         <f>AVERAGE(CONSOLIDADO!G4:G1048576)</f>
-        <v>0.40326457465070203</v>
+        <v>0.39575530586766544</v>
       </c>
       <c r="D4" t="s">
         <v>299</v>
@@ -35430,7 +35430,7 @@
       </c>
       <c r="B12" s="13">
         <f>'FICHA DEL ATLETA'!H6</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -35439,7 +35439,7 @@
       </c>
       <c r="B13" s="13">
         <f>'FICHA DEL ATLETA'!H7</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -35448,7 +35448,7 @@
       </c>
       <c r="B14" s="13">
         <f>'FICHA DEL ATLETA'!H8</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -35457,7 +35457,7 @@
       </c>
       <c r="B15" s="13">
         <f>'FICHA DEL ATLETA'!H9</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -35466,7 +35466,7 @@
       </c>
       <c r="B16" s="13">
         <f>'FICHA DEL ATLETA'!H10</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -35475,7 +35475,7 @@
       </c>
       <c r="B17" s="13">
         <f>'FICHA DEL ATLETA'!H11</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -35484,7 +35484,7 @@
       </c>
       <c r="B18" s="13">
         <f>'FICHA DEL ATLETA'!H12</f>
-        <v>0.88461538461538458</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -35493,7 +35493,7 @@
       </c>
       <c r="B19" s="13">
         <f>'FICHA DEL ATLETA'!H13</f>
-        <v>0.8571428571428571</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -35502,7 +35502,7 @@
       </c>
       <c r="B20" s="13">
         <f>'FICHA DEL ATLETA'!H14</f>
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -35511,7 +35511,7 @@
       </c>
       <c r="B21" s="13">
         <f>'FICHA DEL ATLETA'!H15</f>
-        <v>1</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -35520,7 +35520,7 @@
       </c>
       <c r="B22" s="13">
         <f>'FICHA DEL ATLETA'!H16</f>
-        <v>0.66666666666666663</v>
+        <v>0.6363636363636364</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="B23" s="13">
         <f>'FICHA DEL ATLETA'!H17</f>
-        <v>0.94444444444444442</v>
+        <v>0.9444444444444444</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -35538,7 +35538,7 @@
       </c>
       <c r="B24" s="13">
         <f>'FICHA DEL ATLETA'!H18</f>
-        <v>0.78260869565217395</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -35547,7 +35547,7 @@
       </c>
       <c r="B25" s="13">
         <f>'FICHA DEL ATLETA'!H19</f>
-        <v>0.63636363636363635</v>
+        <v>0.5384615384615384</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -35556,7 +35556,7 @@
       </c>
       <c r="B26" s="13">
         <f>'FICHA DEL ATLETA'!H20</f>
-        <v>0.76923076923076927</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -35565,7 +35565,7 @@
       </c>
       <c r="B27" s="13">
         <f>'FICHA DEL ATLETA'!H21</f>
-        <v>0.82352941176470584</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
   </sheetData>
@@ -35660,8 +35660,8 @@
         <v>9</v>
       </c>
       <c r="G4" s="36">
-        <f t="shared" ref="G4:G33" si="0">IFERROR(C4/(B4-F4),0)</f>
-        <v>0.87984496124031009</v>
+        <f t="shared" ref="G4:G33" si="0">IFERROR(C4/B4,0)</f>
+        <v>0.850187265917603</v>
       </c>
       <c r="H4" s="42" t="str">
         <f>IF(G4&gt;=0.8,"Alto avance",IF(G4&gt;=0.5,"Avance medio",IF(G4&gt;=0.3,"Avance inicial",IF(G4&gt;=0.1,"Base solida","Base inicial"))))</f>
@@ -35694,7 +35694,7 @@
       </c>
       <c r="G5" s="36">
         <f t="shared" si="0"/>
-        <v>0.8132295719844358</v>
+        <v>0.7827715355805244</v>
       </c>
       <c r="H5" s="42" t="str">
         <f t="shared" ref="H5:H33" si="1">IF(G5&gt;=0.8,"Alto avance",IF(G5&gt;=0.5,"Avance medio",IF(G5&gt;=0.3,"Avance inicial",IF(G5&gt;=0.1,"Base solida","Base inicial"))))</f>
@@ -35727,7 +35727,7 @@
       </c>
       <c r="G6" s="36">
         <f t="shared" si="0"/>
-        <v>0.63888888888888884</v>
+        <v>0.602996254681648</v>
       </c>
       <c r="H6" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35760,7 +35760,7 @@
       </c>
       <c r="G7" s="36">
         <f t="shared" si="0"/>
-        <v>0.6731517509727627</v>
+        <v>0.6479400749063671</v>
       </c>
       <c r="H7" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35793,7 +35793,7 @@
       </c>
       <c r="G8" s="36">
         <f t="shared" si="0"/>
-        <v>0.66923076923076918</v>
+        <v>0.651685393258427</v>
       </c>
       <c r="H8" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35826,7 +35826,7 @@
       </c>
       <c r="G9" s="36">
         <f t="shared" si="0"/>
-        <v>0.61153846153846159</v>
+        <v>0.5955056179775281</v>
       </c>
       <c r="H9" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35859,7 +35859,7 @@
       </c>
       <c r="G10" s="36">
         <f t="shared" si="0"/>
-        <v>0.61363636363636365</v>
+        <v>0.6067415730337079</v>
       </c>
       <c r="H10" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35892,7 +35892,7 @@
       </c>
       <c r="G11" s="36">
         <f t="shared" si="0"/>
-        <v>0.55813953488372092</v>
+        <v>0.5393258426966292</v>
       </c>
       <c r="H11" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35925,7 +35925,7 @@
       </c>
       <c r="G12" s="36">
         <f t="shared" si="0"/>
-        <v>0.57198443579766534</v>
+        <v>0.550561797752809</v>
       </c>
       <c r="H12" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35958,7 +35958,7 @@
       </c>
       <c r="G13" s="36">
         <f t="shared" si="0"/>
-        <v>0.45348837209302323</v>
+        <v>0.43820224719101125</v>
       </c>
       <c r="H13" s="42" t="str">
         <f t="shared" si="1"/>
@@ -35991,7 +35991,7 @@
       </c>
       <c r="G14" s="36">
         <f t="shared" si="0"/>
-        <v>0.47565543071161048</v>
+        <v>0.4756554307116105</v>
       </c>
       <c r="H14" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36024,7 +36024,7 @@
       </c>
       <c r="G15" s="36">
         <f t="shared" si="0"/>
-        <v>0.46816479400749061</v>
+        <v>0.4681647940074906</v>
       </c>
       <c r="H15" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36189,7 +36189,7 @@
       </c>
       <c r="G20" s="36">
         <f t="shared" si="0"/>
-        <v>0.28838951310861421</v>
+        <v>0.2883895131086142</v>
       </c>
       <c r="H20" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36255,7 +36255,7 @@
       </c>
       <c r="G22" s="36">
         <f t="shared" si="0"/>
-        <v>0.25939849624060152</v>
+        <v>0.25842696629213485</v>
       </c>
       <c r="H22" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36288,7 +36288,7 @@
       </c>
       <c r="G23" s="36">
         <f t="shared" si="0"/>
-        <v>0.2857142857142857</v>
+        <v>0.2846441947565543</v>
       </c>
       <c r="H23" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36321,7 +36321,7 @@
       </c>
       <c r="G24" s="36">
         <f t="shared" si="0"/>
-        <v>0.25468164794007492</v>
+        <v>0.2546816479400749</v>
       </c>
       <c r="H24" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36354,7 +36354,7 @@
       </c>
       <c r="G25" s="36">
         <f t="shared" si="0"/>
-        <v>0.25468164794007492</v>
+        <v>0.2546816479400749</v>
       </c>
       <c r="H25" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36387,7 +36387,7 @@
       </c>
       <c r="G26" s="36">
         <f t="shared" si="0"/>
-        <v>0.25939849624060152</v>
+        <v>0.25842696629213485</v>
       </c>
       <c r="H26" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36420,7 +36420,7 @@
       </c>
       <c r="G27" s="36">
         <f t="shared" si="0"/>
-        <v>0.24436090225563908</v>
+        <v>0.24344569288389514</v>
       </c>
       <c r="H27" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36453,7 +36453,7 @@
       </c>
       <c r="G28" s="36">
         <f t="shared" si="0"/>
-        <v>0.24812030075187969</v>
+        <v>0.24719101123595505</v>
       </c>
       <c r="H28" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36486,7 +36486,7 @@
       </c>
       <c r="G29" s="36">
         <f t="shared" si="0"/>
-        <v>0.30943396226415093</v>
+        <v>0.30711610486891383</v>
       </c>
       <c r="H29" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36519,7 +36519,7 @@
       </c>
       <c r="G30" s="36">
         <f t="shared" si="0"/>
-        <v>0.23684210526315788</v>
+        <v>0.23595505617977527</v>
       </c>
       <c r="H30" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36585,7 +36585,7 @@
       </c>
       <c r="G32" s="36">
         <f t="shared" si="0"/>
-        <v>9.3632958801498134E-2</v>
+        <v>0.09363295880149813</v>
       </c>
       <c r="H32" s="42" t="str">
         <f t="shared" si="1"/>
@@ -36618,7 +36618,7 @@
       </c>
       <c r="G33" s="45">
         <f t="shared" si="0"/>
-        <v>4.49438202247191E-2</v>
+        <v>0.0449438202247191</v>
       </c>
       <c r="H33" s="46" t="str">
         <f t="shared" si="1"/>

</xml_diff>